<commit_message>
Short Form template: remove conditional formatting
Drops the blank-field hatching on Summary and Setup Information, the
title rule on Summary, and the minimum-thickness highlight on the
Thickness Table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel_templates/paut_corrosion.xlsx
+++ b/excel_templates/paut_corrosion.xlsx
@@ -4303,16 +4303,6 @@
     <mergeCell ref="AA6:AE6"/>
     <mergeCell ref="AF6:AG6"/>
   </mergeCells>
-  <conditionalFormatting sqref="B2 AA5:AO5 L5:U7 AA6 AH6 AO6 AC7 I8 B11:B13 B18 B43:B45">
-    <cfRule type="containsBlanks" dxfId="3" priority="2">
-      <formula>LEN(TRIM(B2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:AO4">
-    <cfRule type="endsWith" dxfId="2" priority="1" operator="endsWith" text="Phased Array Ultrasonic Examinations on Selected Areas On">
-      <formula>RIGHT(B2,LEN("Phased Array Ultrasonic Examinations on Selected Areas On"))="Phased Array Ultrasonic Examinations on Selected Areas On"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" sqref="AA6:AE6" xr:uid="{815EFB7B-C7D4-4002-BB16-07B65D14A11D}">
       <formula1>"100-UT-003, 100-UT-020, 100-UT-021, 100-UT-031"</formula1>
@@ -6756,11 +6746,6 @@
     <mergeCell ref="AB9:AO9"/>
     <mergeCell ref="B9:K9"/>
   </mergeCells>
-  <conditionalFormatting sqref="AG2:AN4 B5:AO6 AJ7:AK7 AN7:AO7 J7:P8 Z7:AB8 AH8:AO8 L9:S9 AB9:AO9">
-    <cfRule type="containsBlanks" dxfId="1" priority="1">
-      <formula>LEN(TRIM(B2))=0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.75" bottom="0.5" header="0.1" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -12351,9 +12336,6 @@
     <mergeCell ref="E2:F4"/>
   </mergeCells>
   <phoneticPr fontId="13" type="noConversion"/>
-  <conditionalFormatting sqref="E20:E37 E6:E18">
-    <cfRule type="top10" dxfId="0" priority="4" bottom="1" rank="1"/>
-  </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.75" bottom="0.5" header="0.1" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>

</xml_diff>